<commit_message>
Modification de la charte exploratoire durant la session
</commit_message>
<xml_diff>
--- a/test-exploratoire/charte-exploratoire.xlsx
+++ b/test-exploratoire/charte-exploratoire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projets\Miniprojet-QA\test-exploratoire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323F0164-463F-4CD8-BAE3-107BAAE87609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA2A7AF-EC7C-45B5-BA69-0D02135CE614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{052C159A-7B27-4D6C-844D-E5DE6F9C3A20}"/>
   </bookViews>
@@ -108,19 +108,21 @@
     <t>Risques à explorer</t>
   </si>
   <si>
-    <t>Disfonctionnement du panier, contraignant l'utilisateur à consulter un site concurrant</t>
-  </si>
-  <si>
     <t>Tâche post-test</t>
   </si>
   <si>
-    <t>Repporter tous les bugs détéctés dans un rapport détaillant le contexte de ces défaillances</t>
-  </si>
-  <si>
     <t>Session n°1</t>
   </si>
   <si>
     <t>Ressources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disfonctionnement du panier, contraignant l'utilisateur à consulter un site concurrant
+</t>
+  </si>
+  <si>
+    <t>Repporter tous les bugs détéctés dans un rapport détaillant le contexte de ces défaillances
+Prendre des captures des différents problèmes rencontrés</t>
   </si>
 </sst>
 </file>
@@ -210,18 +212,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -565,16 +567,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="6"/>
+      <c r="A1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -582,7 +584,7 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -590,7 +592,7 @@
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -598,7 +600,7 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -606,15 +608,15 @@
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3">
-        <v>46175</v>
+      <c r="B6" s="6">
+        <v>46177</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="55.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -622,15 +624,15 @@
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="61.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" ht="57.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -638,7 +640,7 @@
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -646,7 +648,7 @@
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -654,24 +656,24 @@
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>23</v>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>